<commit_message>
fix PR richiesto per accreditamento fse
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#KGPARTNERSSRLXX/KG_Partners_s.r.l/APLAB/V.1/accreditamento_checklist_V8.2.6.xlsx
+++ b/GATEWAY/A1#111#KGPARTNERSSRLXX/KG_Partners_s.r.l/APLAB/V.1/accreditamento_checklist_V8.2.6.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\app\test\php\fse\accreditamento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francesco\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98103A8-4D97-45BC-A34A-BD2D14BEEC0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6DEF5C-36EC-41C8-92A2-D571BA655969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2529,28 +2529,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -2576,6 +2554,28 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
@@ -4054,12 +4054,12 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="52"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="61"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -4080,14 +4080,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="60" t="s">
+      <c r="B3" s="64"/>
+      <c r="C3" s="69" t="s">
         <v>437</v>
       </c>
-      <c r="D3" s="52"/>
+      <c r="D3" s="61"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4108,12 +4108,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="60" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="66"/>
+      <c r="C4" s="69" t="s">
         <v>438</v>
       </c>
-      <c r="D4" s="52"/>
+      <c r="D4" s="61"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -4135,12 +4135,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="58"/>
-      <c r="B5" s="59"/>
-      <c r="C5" s="60" t="s">
+      <c r="A5" s="67"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="69" t="s">
         <v>441</v>
       </c>
-      <c r="D5" s="52"/>
+      <c r="D5" s="61"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -4161,10 +4161,10 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="49"/>
-      <c r="B6" s="50"/>
+      <c r="A6" s="58"/>
+      <c r="B6" s="59"/>
       <c r="C6" s="10"/>
-      <c r="F6" s="61"/>
+      <c r="F6" s="49"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -9621,7 +9621,7 @@
         <v>442</v>
       </c>
       <c r="T151" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U151" s="39"/>
       <c r="V151" s="40"/>
@@ -9684,7 +9684,7 @@
         <v>442</v>
       </c>
       <c r="T152" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U152" s="39"/>
       <c r="V152" s="40"/>
@@ -9743,7 +9743,7 @@
         <v>439</v>
       </c>
       <c r="T153" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U153" s="39"/>
       <c r="V153" s="40"/>
@@ -9806,7 +9806,7 @@
         <v>442</v>
       </c>
       <c r="T154" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U154" s="39"/>
       <c r="V154" s="40"/>
@@ -9869,7 +9869,7 @@
         <v>442</v>
       </c>
       <c r="T155" s="45" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U155" s="39"/>
       <c r="V155" s="40"/>
@@ -9928,7 +9928,7 @@
         <v>442</v>
       </c>
       <c r="T156" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U156" s="39"/>
       <c r="V156" s="40" t="s">
@@ -9938,30 +9938,30 @@
         <v>44</v>
       </c>
     </row>
-    <row r="157" spans="1:23" s="69" customFormat="1" ht="10.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A157" s="62">
+    <row r="157" spans="1:23" s="57" customFormat="1" ht="10.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A157" s="50">
         <v>435</v>
       </c>
-      <c r="B157" s="62" t="s">
-        <v>34</v>
-      </c>
-      <c r="C157" s="63" t="s">
+      <c r="B157" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="C157" s="51" t="s">
         <v>250</v>
       </c>
-      <c r="D157" s="62" t="s">
+      <c r="D157" s="50" t="s">
         <v>260</v>
       </c>
-      <c r="E157" s="64" t="s">
+      <c r="E157" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="F157" s="65">
+      <c r="F157" s="53">
         <v>45827</v>
       </c>
-      <c r="G157" s="65" t="s">
+      <c r="G157" s="53" t="s">
         <v>468</v>
       </c>
-      <c r="H157" s="65"/>
-      <c r="I157" s="66"/>
+      <c r="H157" s="53"/>
+      <c r="I157" s="54"/>
       <c r="J157" s="45" t="s">
         <v>64</v>
       </c>
@@ -9989,10 +9989,10 @@
         <v>442</v>
       </c>
       <c r="T157" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="U157" s="67"/>
-      <c r="V157" s="68" t="s">
+        <v>226</v>
+      </c>
+      <c r="U157" s="55"/>
+      <c r="V157" s="56" t="s">
         <v>440</v>
       </c>
       <c r="W157" s="45" t="s">
@@ -10054,7 +10054,7 @@
         <v>442</v>
       </c>
       <c r="T158" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U158" s="39"/>
       <c r="V158" s="40"/>
@@ -10062,32 +10062,32 @@
         <v>44</v>
       </c>
     </row>
-    <row r="159" spans="1:23" s="69" customFormat="1" ht="10.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A159" s="62">
+    <row r="159" spans="1:23" s="57" customFormat="1" ht="10.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A159" s="50">
         <v>438</v>
       </c>
-      <c r="B159" s="62" t="s">
-        <v>34</v>
-      </c>
-      <c r="C159" s="63" t="s">
+      <c r="B159" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="C159" s="51" t="s">
         <v>250</v>
       </c>
-      <c r="D159" s="62" t="s">
+      <c r="D159" s="50" t="s">
         <v>262</v>
       </c>
-      <c r="E159" s="64" t="s">
+      <c r="E159" s="52" t="s">
         <v>267</v>
       </c>
-      <c r="F159" s="65">
+      <c r="F159" s="53">
         <v>45827</v>
       </c>
-      <c r="G159" s="65" t="s">
+      <c r="G159" s="53" t="s">
         <v>475</v>
       </c>
-      <c r="H159" s="65" t="s">
+      <c r="H159" s="53" t="s">
         <v>476</v>
       </c>
-      <c r="I159" s="66" t="s">
+      <c r="I159" s="54" t="s">
         <v>477</v>
       </c>
       <c r="J159" s="45" t="s">
@@ -10117,10 +10117,10 @@
         <v>442</v>
       </c>
       <c r="T159" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="U159" s="67"/>
-      <c r="V159" s="68"/>
+        <v>226</v>
+      </c>
+      <c r="U159" s="55"/>
+      <c r="V159" s="56"/>
       <c r="W159" s="45" t="s">
         <v>44</v>
       </c>
@@ -10180,7 +10180,7 @@
         <v>442</v>
       </c>
       <c r="T160" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U160" s="39"/>
       <c r="V160" s="40" t="s">
@@ -10245,7 +10245,7 @@
         <v>442</v>
       </c>
       <c r="T161" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U161" s="39"/>
       <c r="V161" s="40"/>
@@ -10308,7 +10308,7 @@
         <v>442</v>
       </c>
       <c r="T162" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U162" s="39"/>
       <c r="V162" s="40"/>
@@ -10371,7 +10371,7 @@
         <v>442</v>
       </c>
       <c r="T163" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U163" s="39"/>
       <c r="V163" s="40" t="s">
@@ -11299,7 +11299,7 @@
         <v>442</v>
       </c>
       <c r="T187" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U187" s="35"/>
       <c r="V187" s="35" t="s">
@@ -11515,7 +11515,7 @@
       <c r="W193" s="9"/>
     </row>
     <row r="194" spans="5:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E194" s="69"/>
+      <c r="E194" s="57"/>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
       <c r="H194" s="6"/>
@@ -17788,12 +17788,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18055,21 +18058,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18094,18 +18103,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>